<commit_message>
Update inventory Excel file
</commit_message>
<xml_diff>
--- a/جرد المواد.xlsx
+++ b/جرد المواد.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\My Drive\InventorySearch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D69FD367-2A14-464A-95CE-40B1D64EF256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5FF9D37-64BD-4D0C-A42A-240746678CFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9897150A-1D18-4DC5-83DE-EA3717EE1A52}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2101" uniqueCount="797">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2098" uniqueCount="796">
   <si>
     <t>3-ديوان</t>
   </si>
@@ -2351,9 +2351,6 @@
   </si>
   <si>
     <t>مجراية بكادوش 50 سم بلاطة جروميكس GROMIX</t>
-  </si>
-  <si>
-    <t>مجراية بكادوش 60 سم بلاطة جروميكس GROMIX</t>
   </si>
   <si>
     <t>مويتر طرمبة غاطسة ليو LEO QDX1.5-17-0.37LA</t>
@@ -2976,7 +2973,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87E5C9A6-5EC3-4592-9122-0E1001CE6231}">
-  <dimension ref="A1:E698"/>
+  <dimension ref="A1:E697"/>
   <sheetFormatPr defaultColWidth="8.69921875" defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.8984375" style="2" bestFit="1" customWidth="1"/>
@@ -3070,7 +3067,7 @@
         <v>39</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="D7" s="13">
         <v>600</v>
@@ -3121,7 +3118,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="D10" s="13">
         <v>500</v>
@@ -4019,13 +4016,13 @@
         <v>572</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C63" s="10" t="s">
         <v>43</v>
       </c>
       <c r="D63" s="13">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="E63" s="1">
         <v>0</v>
@@ -4036,13 +4033,13 @@
         <v>572</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C64" s="10" t="s">
         <v>43</v>
       </c>
       <c r="D64" s="13">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="E64" s="1">
         <v>0</v>
@@ -4172,13 +4169,13 @@
         <v>574</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C72" s="10" t="s">
         <v>47</v>
       </c>
       <c r="D72" s="13">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E72" s="1">
         <v>0</v>
@@ -4189,13 +4186,13 @@
         <v>574</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C73" s="10" t="s">
         <v>47</v>
       </c>
       <c r="D73" s="13">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E73" s="1">
         <v>0</v>
@@ -4444,13 +4441,13 @@
         <v>578</v>
       </c>
       <c r="B88" s="10" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C88" s="10" t="s">
         <v>55</v>
       </c>
       <c r="D88" s="13">
-        <v>1350</v>
+        <v>2725</v>
       </c>
       <c r="E88" s="1">
         <v>0</v>
@@ -4461,13 +4458,13 @@
         <v>578</v>
       </c>
       <c r="B89" s="10" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C89" s="10" t="s">
         <v>55</v>
       </c>
       <c r="D89" s="13">
-        <v>2725</v>
+        <v>1350</v>
       </c>
       <c r="E89" s="1">
         <v>0</v>
@@ -4495,13 +4492,13 @@
         <v>578</v>
       </c>
       <c r="B91" s="10" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C91" s="10" t="s">
         <v>56</v>
       </c>
       <c r="D91" s="13">
-        <v>700</v>
+        <v>75</v>
       </c>
       <c r="E91" s="1">
         <v>0</v>
@@ -4512,13 +4509,13 @@
         <v>578</v>
       </c>
       <c r="B92" s="10" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C92" s="10" t="s">
         <v>56</v>
       </c>
       <c r="D92" s="13">
-        <v>75</v>
+        <v>700</v>
       </c>
       <c r="E92" s="1">
         <v>0</v>
@@ -4685,7 +4682,7 @@
         <v>0</v>
       </c>
       <c r="C102" s="10" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="D102" s="13">
         <v>1</v>
@@ -4787,7 +4784,7 @@
         <v>39</v>
       </c>
       <c r="C108" s="10" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="D108" s="13">
         <v>600</v>
@@ -5158,13 +5155,13 @@
         <v>590</v>
       </c>
       <c r="B130" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C130" s="10" t="s">
         <v>78</v>
       </c>
       <c r="D130" s="13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E130" s="1">
         <v>0</v>
@@ -5175,13 +5172,13 @@
         <v>590</v>
       </c>
       <c r="B131" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C131" s="10" t="s">
         <v>78</v>
       </c>
       <c r="D131" s="13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E131" s="1">
         <v>0</v>
@@ -5192,13 +5189,13 @@
         <v>590</v>
       </c>
       <c r="B132" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C132" s="10" t="s">
         <v>79</v>
       </c>
       <c r="D132" s="13">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E132" s="1">
         <v>0</v>
@@ -5209,13 +5206,13 @@
         <v>590</v>
       </c>
       <c r="B133" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C133" s="10" t="s">
         <v>79</v>
       </c>
       <c r="D133" s="13">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E133" s="1">
         <v>0</v>
@@ -5226,13 +5223,13 @@
         <v>590</v>
       </c>
       <c r="B134" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C134" s="10" t="s">
         <v>80</v>
       </c>
       <c r="D134" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E134" s="1">
         <v>0</v>
@@ -5243,13 +5240,13 @@
         <v>590</v>
       </c>
       <c r="B135" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C135" s="10" t="s">
         <v>80</v>
       </c>
       <c r="D135" s="13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E135" s="1">
         <v>0</v>
@@ -5345,7 +5342,7 @@
         <v>590</v>
       </c>
       <c r="B141" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C141" s="10" t="s">
         <v>84</v>
@@ -5362,7 +5359,7 @@
         <v>590</v>
       </c>
       <c r="B142" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C142" s="10" t="s">
         <v>84</v>
@@ -5498,13 +5495,13 @@
         <v>590</v>
       </c>
       <c r="B150" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C150" s="10" t="s">
         <v>92</v>
       </c>
       <c r="D150" s="13">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E150" s="1">
         <v>0</v>
@@ -5515,13 +5512,13 @@
         <v>590</v>
       </c>
       <c r="B151" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C151" s="10" t="s">
         <v>92</v>
       </c>
       <c r="D151" s="13">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E151" s="1">
         <v>0</v>
@@ -6110,13 +6107,13 @@
         <v>584</v>
       </c>
       <c r="B186" s="10" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="C186" s="10" t="s">
         <v>699</v>
       </c>
       <c r="D186" s="13">
-        <v>1920</v>
+        <v>400</v>
       </c>
       <c r="E186" s="1">
         <v>0</v>
@@ -6127,13 +6124,13 @@
         <v>584</v>
       </c>
       <c r="B187" s="10" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="C187" s="10" t="s">
         <v>699</v>
       </c>
       <c r="D187" s="13">
-        <v>400</v>
+        <v>1920</v>
       </c>
       <c r="E187" s="1">
         <v>0</v>
@@ -6144,13 +6141,13 @@
         <v>584</v>
       </c>
       <c r="B188" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C188" s="10" t="s">
         <v>497</v>
       </c>
       <c r="D188" s="13">
-        <v>1600</v>
+        <v>240</v>
       </c>
       <c r="E188" s="1">
         <v>0</v>
@@ -6161,13 +6158,13 @@
         <v>584</v>
       </c>
       <c r="B189" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C189" s="10" t="s">
         <v>497</v>
       </c>
       <c r="D189" s="13">
-        <v>240</v>
+        <v>1600</v>
       </c>
       <c r="E189" s="1">
         <v>0</v>
@@ -6252,7 +6249,7 @@
         <v>701</v>
       </c>
       <c r="D194" s="13">
-        <v>2880</v>
+        <v>2720</v>
       </c>
       <c r="E194" s="1">
         <v>0</v>
@@ -6283,7 +6280,7 @@
         <v>39</v>
       </c>
       <c r="C196" s="10" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="D196" s="13">
         <v>2040</v>
@@ -6742,7 +6739,7 @@
         <v>39</v>
       </c>
       <c r="C223" s="10" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="D223" s="13">
         <v>100</v>
@@ -7099,7 +7096,7 @@
         <v>39</v>
       </c>
       <c r="C244" s="10" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="D244" s="13">
         <v>800</v>
@@ -7164,13 +7161,13 @@
         <v>613</v>
       </c>
       <c r="B248" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C248" s="10" t="s">
         <v>146</v>
       </c>
       <c r="D248" s="13">
-        <v>95</v>
+        <v>150</v>
       </c>
       <c r="E248" s="1">
         <v>0</v>
@@ -7181,13 +7178,13 @@
         <v>613</v>
       </c>
       <c r="B249" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C249" s="10" t="s">
         <v>146</v>
       </c>
       <c r="D249" s="13">
-        <v>150</v>
+        <v>95</v>
       </c>
       <c r="E249" s="1">
         <v>0</v>
@@ -7266,13 +7263,13 @@
         <v>613</v>
       </c>
       <c r="B254" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C254" s="10" t="s">
         <v>148</v>
       </c>
       <c r="D254" s="13">
-        <v>520</v>
+        <v>600</v>
       </c>
       <c r="E254" s="1">
         <v>0</v>
@@ -7283,13 +7280,13 @@
         <v>613</v>
       </c>
       <c r="B255" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C255" s="10" t="s">
         <v>148</v>
       </c>
       <c r="D255" s="13">
-        <v>600</v>
+        <v>520</v>
       </c>
       <c r="E255" s="1">
         <v>0</v>
@@ -7493,7 +7490,7 @@
         <v>158</v>
       </c>
       <c r="D267" s="13">
-        <v>269</v>
+        <v>249</v>
       </c>
       <c r="E267" s="1">
         <v>0</v>
@@ -7864,7 +7861,7 @@
         <v>0</v>
       </c>
       <c r="C289" s="10" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="D289" s="13">
         <v>30</v>
@@ -7884,7 +7881,7 @@
         <v>740</v>
       </c>
       <c r="D290" s="13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E290" s="1">
         <v>0</v>
@@ -8286,13 +8283,13 @@
         <v>620</v>
       </c>
       <c r="B314" s="10" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="C314" s="10" t="s">
         <v>181</v>
       </c>
       <c r="D314" s="13">
-        <v>800</v>
+        <v>125</v>
       </c>
       <c r="E314" s="1">
         <v>0</v>
@@ -8320,13 +8317,13 @@
         <v>620</v>
       </c>
       <c r="B316" s="10" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="C316" s="10" t="s">
         <v>181</v>
       </c>
       <c r="D316" s="13">
-        <v>125</v>
+        <v>800</v>
       </c>
       <c r="E316" s="1">
         <v>0</v>
@@ -8694,13 +8691,13 @@
         <v>628</v>
       </c>
       <c r="B338" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C338" s="10" t="s">
         <v>188</v>
       </c>
       <c r="D338" s="13">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="E338" s="1">
         <v>0</v>
@@ -8711,13 +8708,13 @@
         <v>628</v>
       </c>
       <c r="B339" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C339" s="10" t="s">
         <v>188</v>
       </c>
       <c r="D339" s="13">
-        <v>300</v>
+        <v>280</v>
       </c>
       <c r="E339" s="1">
         <v>0</v>
@@ -9258,7 +9255,7 @@
         <v>0</v>
       </c>
       <c r="C371" s="10" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="D371" s="13">
         <v>24</v>
@@ -9612,13 +9609,13 @@
         <v>636</v>
       </c>
       <c r="B392" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C392" s="10" t="s">
         <v>217</v>
       </c>
       <c r="D392" s="13">
-        <v>360</v>
+        <v>200</v>
       </c>
       <c r="E392" s="1">
         <v>0</v>
@@ -9629,13 +9626,13 @@
         <v>636</v>
       </c>
       <c r="B393" s="10" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C393" s="10" t="s">
         <v>217</v>
       </c>
       <c r="D393" s="13">
-        <v>200</v>
+        <v>2550</v>
       </c>
       <c r="E393" s="1">
         <v>0</v>
@@ -9646,13 +9643,13 @@
         <v>636</v>
       </c>
       <c r="B394" s="10" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="C394" s="10" t="s">
         <v>217</v>
       </c>
       <c r="D394" s="13">
-        <v>2550</v>
+        <v>360</v>
       </c>
       <c r="E394" s="1">
         <v>0</v>
@@ -10105,13 +10102,13 @@
         <v>644</v>
       </c>
       <c r="B421" s="10" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C421" s="10" t="s">
         <v>233</v>
       </c>
       <c r="D421" s="13">
-        <v>1775</v>
+        <v>300</v>
       </c>
       <c r="E421" s="1">
         <v>0</v>
@@ -10122,13 +10119,13 @@
         <v>644</v>
       </c>
       <c r="B422" s="10" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C422" s="10" t="s">
         <v>233</v>
       </c>
       <c r="D422" s="13">
-        <v>300</v>
+        <v>1775</v>
       </c>
       <c r="E422" s="1">
         <v>0</v>
@@ -10723,7 +10720,7 @@
         <v>762</v>
       </c>
       <c r="D457" s="13">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E457" s="1">
         <v>0</v>
@@ -10740,7 +10737,7 @@
         <v>763</v>
       </c>
       <c r="D458" s="13">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E458" s="1">
         <v>0</v>
@@ -10748,16 +10745,16 @@
     </row>
     <row r="459" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A459" s="10" t="s">
-        <v>592</v>
+        <v>583</v>
       </c>
       <c r="B459" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C459" s="10" t="s">
-        <v>764</v>
+        <v>694</v>
       </c>
       <c r="D459" s="13">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E459" s="1">
         <v>0</v>
@@ -10771,10 +10768,10 @@
         <v>0</v>
       </c>
       <c r="C460" s="10" t="s">
-        <v>694</v>
+        <v>474</v>
       </c>
       <c r="D460" s="13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E460" s="1">
         <v>0</v>
@@ -10782,16 +10779,16 @@
     </row>
     <row r="461" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A461" s="10" t="s">
-        <v>583</v>
+        <v>652</v>
       </c>
       <c r="B461" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C461" s="10" t="s">
-        <v>474</v>
+        <v>254</v>
       </c>
       <c r="D461" s="13">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="E461" s="1">
         <v>0</v>
@@ -10799,16 +10796,16 @@
     </row>
     <row r="462" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A462" s="10" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B462" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C462" s="10" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D462" s="13">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="E462" s="1">
         <v>0</v>
@@ -10819,13 +10816,13 @@
         <v>653</v>
       </c>
       <c r="B463" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C463" s="10" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D463" s="13">
-        <v>47</v>
+        <v>830</v>
       </c>
       <c r="E463" s="1">
         <v>0</v>
@@ -10839,10 +10836,10 @@
         <v>39</v>
       </c>
       <c r="C464" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D464" s="13">
-        <v>830</v>
+        <v>850</v>
       </c>
       <c r="E464" s="1">
         <v>0</v>
@@ -10856,10 +10853,10 @@
         <v>39</v>
       </c>
       <c r="C465" s="10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D465" s="13">
-        <v>850</v>
+        <v>1250</v>
       </c>
       <c r="E465" s="1">
         <v>0</v>
@@ -10873,10 +10870,10 @@
         <v>39</v>
       </c>
       <c r="C466" s="10" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D466" s="13">
-        <v>1250</v>
+        <v>400</v>
       </c>
       <c r="E466" s="1">
         <v>0</v>
@@ -10884,16 +10881,16 @@
     </row>
     <row r="467" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A467" s="10" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B467" s="10" t="s">
         <v>39</v>
       </c>
       <c r="C467" s="10" t="s">
-        <v>259</v>
+        <v>773</v>
       </c>
       <c r="D467" s="13">
-        <v>400</v>
+        <v>3760</v>
       </c>
       <c r="E467" s="1">
         <v>0</v>
@@ -10904,13 +10901,13 @@
         <v>652</v>
       </c>
       <c r="B468" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C468" s="10" t="s">
-        <v>774</v>
+        <v>260</v>
       </c>
       <c r="D468" s="13">
-        <v>3760</v>
+        <v>779</v>
       </c>
       <c r="E468" s="1">
         <v>0</v>
@@ -10935,16 +10932,16 @@
     </row>
     <row r="470" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A470" s="10" t="s">
-        <v>652</v>
+        <v>552</v>
       </c>
       <c r="B470" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C470" s="10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D470" s="13">
-        <v>779</v>
+        <v>273</v>
       </c>
       <c r="E470" s="1">
         <v>0</v>
@@ -10952,16 +10949,16 @@
     </row>
     <row r="471" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A471" s="10" t="s">
-        <v>552</v>
+        <v>652</v>
       </c>
       <c r="B471" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C471" s="10" t="s">
-        <v>261</v>
+        <v>774</v>
       </c>
       <c r="D471" s="13">
-        <v>273</v>
+        <v>1632</v>
       </c>
       <c r="E471" s="1">
         <v>0</v>
@@ -10969,16 +10966,16 @@
     </row>
     <row r="472" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A472" s="10" t="s">
-        <v>652</v>
+        <v>568</v>
       </c>
       <c r="B472" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C472" s="10" t="s">
-        <v>775</v>
+        <v>262</v>
       </c>
       <c r="D472" s="13">
-        <v>1632</v>
+        <v>3</v>
       </c>
       <c r="E472" s="1">
         <v>0</v>
@@ -10992,10 +10989,10 @@
         <v>0</v>
       </c>
       <c r="C473" s="10" t="s">
-        <v>262</v>
+        <v>502</v>
       </c>
       <c r="D473" s="13">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="E473" s="1">
         <v>0</v>
@@ -11003,16 +11000,16 @@
     </row>
     <row r="474" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A474" s="10" t="s">
-        <v>568</v>
+        <v>606</v>
       </c>
       <c r="B474" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C474" s="10" t="s">
-        <v>502</v>
+        <v>263</v>
       </c>
       <c r="D474" s="13">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="E474" s="1">
         <v>0</v>
@@ -11026,10 +11023,10 @@
         <v>0</v>
       </c>
       <c r="C475" s="10" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D475" s="13">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E475" s="1">
         <v>0</v>
@@ -11040,13 +11037,13 @@
         <v>606</v>
       </c>
       <c r="B476" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C476" s="10" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D476" s="13">
-        <v>6</v>
+        <v>840</v>
       </c>
       <c r="E476" s="1">
         <v>0</v>
@@ -11060,10 +11057,10 @@
         <v>39</v>
       </c>
       <c r="C477" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D477" s="13">
-        <v>840</v>
+        <v>10</v>
       </c>
       <c r="E477" s="1">
         <v>0</v>
@@ -11077,7 +11074,7 @@
         <v>39</v>
       </c>
       <c r="C478" s="10" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D478" s="13">
         <v>10</v>
@@ -11094,10 +11091,10 @@
         <v>39</v>
       </c>
       <c r="C479" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D479" s="13">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="E479" s="1">
         <v>0</v>
@@ -11111,10 +11108,10 @@
         <v>39</v>
       </c>
       <c r="C480" s="10" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D480" s="13">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="E480" s="1">
         <v>0</v>
@@ -11128,10 +11125,10 @@
         <v>39</v>
       </c>
       <c r="C481" s="10" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D481" s="13">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="E481" s="1">
         <v>0</v>
@@ -11145,10 +11142,10 @@
         <v>39</v>
       </c>
       <c r="C482" s="10" t="s">
-        <v>270</v>
+        <v>418</v>
       </c>
       <c r="D482" s="13">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E482" s="1">
         <v>0</v>
@@ -11156,16 +11153,16 @@
     </row>
     <row r="483" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A483" s="10" t="s">
-        <v>606</v>
+        <v>549</v>
       </c>
       <c r="B483" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C483" s="10" t="s">
-        <v>418</v>
+        <v>271</v>
       </c>
       <c r="D483" s="13">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="E483" s="1">
         <v>0</v>
@@ -11173,16 +11170,16 @@
     </row>
     <row r="484" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A484" s="10" t="s">
-        <v>549</v>
+        <v>652</v>
       </c>
       <c r="B484" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C484" s="10" t="s">
-        <v>271</v>
+        <v>775</v>
       </c>
       <c r="D484" s="13">
-        <v>75</v>
+        <v>575</v>
       </c>
       <c r="E484" s="1">
         <v>0</v>
@@ -11199,7 +11196,7 @@
         <v>776</v>
       </c>
       <c r="D485" s="13">
-        <v>575</v>
+        <v>9500</v>
       </c>
       <c r="E485" s="1">
         <v>0</v>
@@ -11216,7 +11213,7 @@
         <v>777</v>
       </c>
       <c r="D486" s="13">
-        <v>9500</v>
+        <v>575</v>
       </c>
       <c r="E486" s="1">
         <v>0</v>
@@ -11227,13 +11224,13 @@
         <v>652</v>
       </c>
       <c r="B487" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C487" s="10" t="s">
-        <v>778</v>
+        <v>272</v>
       </c>
       <c r="D487" s="13">
-        <v>575</v>
+        <v>40</v>
       </c>
       <c r="E487" s="1">
         <v>0</v>
@@ -11244,13 +11241,13 @@
         <v>652</v>
       </c>
       <c r="B488" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C488" s="10" t="s">
-        <v>272</v>
+        <v>778</v>
       </c>
       <c r="D488" s="13">
-        <v>40</v>
+        <v>5000</v>
       </c>
       <c r="E488" s="1">
         <v>0</v>
@@ -11258,16 +11255,16 @@
     </row>
     <row r="489" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A489" s="10" t="s">
-        <v>652</v>
+        <v>551</v>
       </c>
       <c r="B489" s="10" t="s">
         <v>39</v>
       </c>
       <c r="C489" s="10" t="s">
-        <v>779</v>
+        <v>410</v>
       </c>
       <c r="D489" s="13">
-        <v>5000</v>
+        <v>16400</v>
       </c>
       <c r="E489" s="1">
         <v>0</v>
@@ -11275,16 +11272,16 @@
     </row>
     <row r="490" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A490" s="10" t="s">
-        <v>551</v>
+        <v>565</v>
       </c>
       <c r="B490" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C490" s="10" t="s">
-        <v>410</v>
+        <v>273</v>
       </c>
       <c r="D490" s="13">
-        <v>16400</v>
+        <v>1</v>
       </c>
       <c r="E490" s="1">
         <v>0</v>
@@ -11298,10 +11295,10 @@
         <v>0</v>
       </c>
       <c r="C491" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D491" s="13">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E491" s="1">
         <v>0</v>
@@ -11315,10 +11312,10 @@
         <v>0</v>
       </c>
       <c r="C492" s="10" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D492" s="13">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E492" s="1">
         <v>0</v>
@@ -11332,10 +11329,10 @@
         <v>0</v>
       </c>
       <c r="C493" s="10" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D493" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E493" s="1">
         <v>0</v>
@@ -11349,7 +11346,7 @@
         <v>0</v>
       </c>
       <c r="C494" s="10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D494" s="13">
         <v>1</v>
@@ -11366,7 +11363,7 @@
         <v>0</v>
       </c>
       <c r="C495" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D495" s="13">
         <v>1</v>
@@ -11383,7 +11380,7 @@
         <v>0</v>
       </c>
       <c r="C496" s="10" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D496" s="13">
         <v>1</v>
@@ -11400,10 +11397,10 @@
         <v>0</v>
       </c>
       <c r="C497" s="10" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D497" s="13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E497" s="1">
         <v>0</v>
@@ -11417,10 +11414,10 @@
         <v>0</v>
       </c>
       <c r="C498" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D498" s="13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E498" s="1">
         <v>0</v>
@@ -11434,10 +11431,10 @@
         <v>0</v>
       </c>
       <c r="C499" s="10" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D499" s="13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E499" s="1">
         <v>0</v>
@@ -11445,16 +11442,16 @@
     </row>
     <row r="500" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A500" s="10" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B500" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C500" s="10" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D500" s="13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E500" s="1">
         <v>0</v>
@@ -11462,16 +11459,16 @@
     </row>
     <row r="501" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A501" s="10" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B501" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C501" s="10" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D501" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E501" s="1">
         <v>0</v>
@@ -11485,10 +11482,10 @@
         <v>0</v>
       </c>
       <c r="C502" s="10" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D502" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E502" s="1">
         <v>0</v>
@@ -11496,13 +11493,13 @@
     </row>
     <row r="503" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A503" s="10" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B503" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C503" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D503" s="13">
         <v>1</v>
@@ -11513,13 +11510,13 @@
     </row>
     <row r="504" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A504" s="10" t="s">
-        <v>566</v>
+        <v>549</v>
       </c>
       <c r="B504" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C504" s="10" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D504" s="13">
         <v>1</v>
@@ -11530,13 +11527,13 @@
     </row>
     <row r="505" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A505" s="10" t="s">
-        <v>549</v>
+        <v>611</v>
       </c>
       <c r="B505" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C505" s="10" t="s">
-        <v>287</v>
+        <v>478</v>
       </c>
       <c r="D505" s="13">
         <v>1</v>
@@ -11553,7 +11550,7 @@
         <v>0</v>
       </c>
       <c r="C506" s="10" t="s">
-        <v>478</v>
+        <v>288</v>
       </c>
       <c r="D506" s="13">
         <v>1</v>
@@ -11564,16 +11561,16 @@
     </row>
     <row r="507" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A507" s="10" t="s">
-        <v>611</v>
+        <v>549</v>
       </c>
       <c r="B507" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C507" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D507" s="13">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E507" s="1">
         <v>0</v>
@@ -11581,13 +11578,13 @@
     </row>
     <row r="508" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A508" s="10" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="B508" s="10" t="s">
-        <v>0</v>
+        <v>515</v>
       </c>
       <c r="C508" s="10" t="s">
-        <v>289</v>
+        <v>706</v>
       </c>
       <c r="D508" s="13">
         <v>7</v>
@@ -11604,10 +11601,10 @@
         <v>515</v>
       </c>
       <c r="C509" s="10" t="s">
-        <v>706</v>
+        <v>676</v>
       </c>
       <c r="D509" s="13">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E509" s="1">
         <v>0</v>
@@ -11621,10 +11618,10 @@
         <v>515</v>
       </c>
       <c r="C510" s="10" t="s">
-        <v>676</v>
+        <v>754</v>
       </c>
       <c r="D510" s="13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E510" s="1">
         <v>0</v>
@@ -11638,10 +11635,10 @@
         <v>515</v>
       </c>
       <c r="C511" s="10" t="s">
-        <v>754</v>
+        <v>516</v>
       </c>
       <c r="D511" s="13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E511" s="1">
         <v>0</v>
@@ -11655,10 +11652,10 @@
         <v>515</v>
       </c>
       <c r="C512" s="10" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D512" s="13">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E512" s="1">
         <v>0</v>
@@ -11666,16 +11663,16 @@
     </row>
     <row r="513" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A513" s="10" t="s">
-        <v>555</v>
+        <v>655</v>
       </c>
       <c r="B513" s="10" t="s">
-        <v>515</v>
+        <v>0</v>
       </c>
       <c r="C513" s="10" t="s">
-        <v>517</v>
+        <v>693</v>
       </c>
       <c r="D513" s="13">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="E513" s="1">
         <v>0</v>
@@ -11683,16 +11680,16 @@
     </row>
     <row r="514" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A514" s="10" t="s">
-        <v>655</v>
+        <v>555</v>
       </c>
       <c r="B514" s="10" t="s">
-        <v>0</v>
+        <v>515</v>
       </c>
       <c r="C514" s="10" t="s">
-        <v>693</v>
+        <v>518</v>
       </c>
       <c r="D514" s="13">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="E514" s="1">
         <v>0</v>
@@ -11706,10 +11703,10 @@
         <v>515</v>
       </c>
       <c r="C515" s="10" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="D515" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E515" s="1">
         <v>0</v>
@@ -11723,10 +11720,10 @@
         <v>515</v>
       </c>
       <c r="C516" s="10" t="s">
-        <v>519</v>
+        <v>791</v>
       </c>
       <c r="D516" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E516" s="1">
         <v>0</v>
@@ -11740,10 +11737,10 @@
         <v>515</v>
       </c>
       <c r="C517" s="10" t="s">
-        <v>792</v>
+        <v>695</v>
       </c>
       <c r="D517" s="13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E517" s="1">
         <v>0</v>
@@ -11757,7 +11754,7 @@
         <v>515</v>
       </c>
       <c r="C518" s="10" t="s">
-        <v>695</v>
+        <v>707</v>
       </c>
       <c r="D518" s="13">
         <v>2</v>
@@ -11774,10 +11771,10 @@
         <v>515</v>
       </c>
       <c r="C519" s="10" t="s">
-        <v>707</v>
+        <v>520</v>
       </c>
       <c r="D519" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E519" s="1">
         <v>0</v>
@@ -11791,7 +11788,7 @@
         <v>515</v>
       </c>
       <c r="C520" s="10" t="s">
-        <v>520</v>
+        <v>757</v>
       </c>
       <c r="D520" s="13">
         <v>1</v>
@@ -11805,10 +11802,10 @@
         <v>555</v>
       </c>
       <c r="B521" s="10" t="s">
-        <v>515</v>
+        <v>0</v>
       </c>
       <c r="C521" s="10" t="s">
-        <v>757</v>
+        <v>290</v>
       </c>
       <c r="D521" s="13">
         <v>1</v>
@@ -11819,13 +11816,13 @@
     </row>
     <row r="522" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A522" s="10" t="s">
-        <v>555</v>
+        <v>655</v>
       </c>
       <c r="B522" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C522" s="10" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D522" s="13">
         <v>1</v>
@@ -11842,10 +11839,10 @@
         <v>0</v>
       </c>
       <c r="C523" s="10" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D523" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E523" s="1">
         <v>0</v>
@@ -11859,10 +11856,10 @@
         <v>0</v>
       </c>
       <c r="C524" s="10" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D524" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E524" s="1">
         <v>0</v>
@@ -11876,7 +11873,7 @@
         <v>0</v>
       </c>
       <c r="C525" s="10" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D525" s="13">
         <v>1</v>
@@ -11893,7 +11890,7 @@
         <v>0</v>
       </c>
       <c r="C526" s="10" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D526" s="13">
         <v>1</v>
@@ -11910,7 +11907,7 @@
         <v>0</v>
       </c>
       <c r="C527" s="10" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D527" s="13">
         <v>1</v>
@@ -11927,10 +11924,10 @@
         <v>0</v>
       </c>
       <c r="C528" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D528" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E528" s="1">
         <v>0</v>
@@ -11938,13 +11935,13 @@
     </row>
     <row r="529" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A529" s="10" t="s">
-        <v>655</v>
+        <v>555</v>
       </c>
       <c r="B529" s="10" t="s">
-        <v>0</v>
+        <v>515</v>
       </c>
       <c r="C529" s="10" t="s">
-        <v>297</v>
+        <v>521</v>
       </c>
       <c r="D529" s="13">
         <v>2</v>
@@ -11961,10 +11958,10 @@
         <v>515</v>
       </c>
       <c r="C530" s="10" t="s">
-        <v>521</v>
+        <v>698</v>
       </c>
       <c r="D530" s="13">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E530" s="1">
         <v>0</v>
@@ -11978,10 +11975,10 @@
         <v>515</v>
       </c>
       <c r="C531" s="10" t="s">
-        <v>698</v>
+        <v>522</v>
       </c>
       <c r="D531" s="13">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E531" s="1">
         <v>0</v>
@@ -11995,10 +11992,10 @@
         <v>515</v>
       </c>
       <c r="C532" s="10" t="s">
-        <v>522</v>
+        <v>692</v>
       </c>
       <c r="D532" s="13">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E532" s="1">
         <v>0</v>
@@ -12012,10 +12009,10 @@
         <v>515</v>
       </c>
       <c r="C533" s="10" t="s">
-        <v>692</v>
+        <v>705</v>
       </c>
       <c r="D533" s="13">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E533" s="1">
         <v>0</v>
@@ -12029,10 +12026,10 @@
         <v>515</v>
       </c>
       <c r="C534" s="10" t="s">
-        <v>705</v>
+        <v>750</v>
       </c>
       <c r="D534" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E534" s="1">
         <v>0</v>
@@ -12040,16 +12037,16 @@
     </row>
     <row r="535" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A535" s="10" t="s">
-        <v>555</v>
+        <v>743</v>
       </c>
       <c r="B535" s="10" t="s">
-        <v>515</v>
+        <v>0</v>
       </c>
       <c r="C535" s="10" t="s">
-        <v>750</v>
+        <v>744</v>
       </c>
       <c r="D535" s="13">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E535" s="1">
         <v>0</v>
@@ -12057,16 +12054,16 @@
     </row>
     <row r="536" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A536" s="10" t="s">
-        <v>743</v>
+        <v>557</v>
       </c>
       <c r="B536" s="10" t="s">
-        <v>0</v>
+        <v>515</v>
       </c>
       <c r="C536" s="10" t="s">
-        <v>744</v>
+        <v>696</v>
       </c>
       <c r="D536" s="13">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E536" s="1">
         <v>0</v>
@@ -12080,7 +12077,7 @@
         <v>515</v>
       </c>
       <c r="C537" s="10" t="s">
-        <v>696</v>
+        <v>523</v>
       </c>
       <c r="D537" s="13">
         <v>1</v>
@@ -12091,13 +12088,13 @@
     </row>
     <row r="538" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A538" s="10" t="s">
-        <v>557</v>
+        <v>611</v>
       </c>
       <c r="B538" s="10" t="s">
         <v>515</v>
       </c>
       <c r="C538" s="10" t="s">
-        <v>523</v>
+        <v>736</v>
       </c>
       <c r="D538" s="13">
         <v>1</v>
@@ -12114,10 +12111,10 @@
         <v>515</v>
       </c>
       <c r="C539" s="10" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="D539" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E539" s="1">
         <v>0</v>
@@ -12125,16 +12122,16 @@
     </row>
     <row r="540" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A540" s="10" t="s">
-        <v>611</v>
+        <v>654</v>
       </c>
       <c r="B540" s="10" t="s">
         <v>515</v>
       </c>
       <c r="C540" s="10" t="s">
-        <v>737</v>
+        <v>524</v>
       </c>
       <c r="D540" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E540" s="1">
         <v>0</v>
@@ -12148,7 +12145,7 @@
         <v>515</v>
       </c>
       <c r="C541" s="10" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="D541" s="13">
         <v>1</v>
@@ -12159,13 +12156,13 @@
     </row>
     <row r="542" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A542" s="10" t="s">
-        <v>654</v>
+        <v>557</v>
       </c>
       <c r="B542" s="10" t="s">
         <v>515</v>
       </c>
       <c r="C542" s="10" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="D542" s="13">
         <v>1</v>
@@ -12182,7 +12179,7 @@
         <v>515</v>
       </c>
       <c r="C543" s="10" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="D543" s="13">
         <v>1</v>
@@ -12199,7 +12196,7 @@
         <v>515</v>
       </c>
       <c r="C544" s="10" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="D544" s="13">
         <v>1</v>
@@ -12216,10 +12213,10 @@
         <v>515</v>
       </c>
       <c r="C545" s="10" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="D545" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E545" s="1">
         <v>0</v>
@@ -12233,10 +12230,10 @@
         <v>515</v>
       </c>
       <c r="C546" s="10" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D546" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E546" s="1">
         <v>0</v>
@@ -12244,16 +12241,16 @@
     </row>
     <row r="547" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A547" s="10" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="B547" s="10" t="s">
         <v>515</v>
       </c>
       <c r="C547" s="10" t="s">
-        <v>530</v>
+        <v>545</v>
       </c>
       <c r="D547" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E547" s="1">
         <v>0</v>
@@ -12267,10 +12264,10 @@
         <v>515</v>
       </c>
       <c r="C548" s="10" t="s">
-        <v>545</v>
+        <v>531</v>
       </c>
       <c r="D548" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E548" s="1">
         <v>0</v>
@@ -12284,7 +12281,7 @@
         <v>515</v>
       </c>
       <c r="C549" s="10" t="s">
-        <v>531</v>
+        <v>546</v>
       </c>
       <c r="D549" s="13">
         <v>1</v>
@@ -12301,7 +12298,7 @@
         <v>515</v>
       </c>
       <c r="C550" s="10" t="s">
-        <v>546</v>
+        <v>532</v>
       </c>
       <c r="D550" s="13">
         <v>1</v>
@@ -12312,13 +12309,13 @@
     </row>
     <row r="551" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A551" s="10" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B551" s="10" t="s">
         <v>515</v>
       </c>
       <c r="C551" s="10" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="D551" s="13">
         <v>1</v>
@@ -12335,7 +12332,7 @@
         <v>515</v>
       </c>
       <c r="C552" s="10" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="D552" s="13">
         <v>1</v>
@@ -12346,13 +12343,13 @@
     </row>
     <row r="553" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A553" s="10" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="B553" s="10" t="s">
         <v>515</v>
       </c>
       <c r="C553" s="10" t="s">
-        <v>534</v>
+        <v>547</v>
       </c>
       <c r="D553" s="13">
         <v>1</v>
@@ -12369,7 +12366,7 @@
         <v>515</v>
       </c>
       <c r="C554" s="10" t="s">
-        <v>547</v>
+        <v>535</v>
       </c>
       <c r="D554" s="13">
         <v>1</v>
@@ -12386,10 +12383,10 @@
         <v>515</v>
       </c>
       <c r="C555" s="10" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="D555" s="13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E555" s="1">
         <v>0</v>
@@ -12403,10 +12400,10 @@
         <v>515</v>
       </c>
       <c r="C556" s="10" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D556" s="13">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E556" s="1">
         <v>0</v>
@@ -12420,10 +12417,10 @@
         <v>515</v>
       </c>
       <c r="C557" s="10" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="D557" s="13">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E557" s="1">
         <v>0</v>
@@ -12437,10 +12434,10 @@
         <v>515</v>
       </c>
       <c r="C558" s="10" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="D558" s="13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E558" s="1">
         <v>0</v>
@@ -12454,10 +12451,10 @@
         <v>515</v>
       </c>
       <c r="C559" s="10" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="D559" s="13">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E559" s="1">
         <v>0</v>
@@ -12465,16 +12462,16 @@
     </row>
     <row r="560" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A560" s="10" t="s">
-        <v>555</v>
+        <v>611</v>
       </c>
       <c r="B560" s="10" t="s">
         <v>515</v>
       </c>
       <c r="C560" s="10" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="D560" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E560" s="1">
         <v>0</v>
@@ -12482,16 +12479,16 @@
     </row>
     <row r="561" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A561" s="10" t="s">
-        <v>611</v>
+        <v>655</v>
       </c>
       <c r="B561" s="10" t="s">
-        <v>515</v>
+        <v>0</v>
       </c>
       <c r="C561" s="10" t="s">
-        <v>541</v>
+        <v>298</v>
       </c>
       <c r="D561" s="13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E561" s="1">
         <v>0</v>
@@ -12499,13 +12496,13 @@
     </row>
     <row r="562" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A562" s="10" t="s">
-        <v>655</v>
+        <v>555</v>
       </c>
       <c r="B562" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C562" s="10" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D562" s="13">
         <v>1</v>
@@ -12522,7 +12519,7 @@
         <v>0</v>
       </c>
       <c r="C563" s="10" t="s">
-        <v>299</v>
+        <v>486</v>
       </c>
       <c r="D563" s="13">
         <v>1</v>
@@ -12539,10 +12536,10 @@
         <v>0</v>
       </c>
       <c r="C564" s="10" t="s">
-        <v>486</v>
+        <v>300</v>
       </c>
       <c r="D564" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E564" s="1">
         <v>0</v>
@@ -12567,13 +12564,13 @@
     </row>
     <row r="566" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A566" s="10" t="s">
-        <v>555</v>
+        <v>611</v>
       </c>
       <c r="B566" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C566" s="10" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D566" s="13">
         <v>2</v>
@@ -12590,10 +12587,10 @@
         <v>0</v>
       </c>
       <c r="C567" s="10" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D567" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E567" s="1">
         <v>0</v>
@@ -12607,7 +12604,7 @@
         <v>0</v>
       </c>
       <c r="C568" s="10" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D568" s="13">
         <v>1</v>
@@ -12618,13 +12615,13 @@
     </row>
     <row r="569" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A569" s="10" t="s">
-        <v>611</v>
+        <v>557</v>
       </c>
       <c r="B569" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C569" s="10" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D569" s="13">
         <v>1</v>
@@ -12641,7 +12638,7 @@
         <v>0</v>
       </c>
       <c r="C570" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D570" s="13">
         <v>1</v>
@@ -12652,16 +12649,16 @@
     </row>
     <row r="571" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A571" s="10" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="B571" s="10" t="s">
-        <v>0</v>
+        <v>515</v>
       </c>
       <c r="C571" s="10" t="s">
-        <v>305</v>
+        <v>680</v>
       </c>
       <c r="D571" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E571" s="1">
         <v>0</v>
@@ -12675,10 +12672,10 @@
         <v>515</v>
       </c>
       <c r="C572" s="10" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="D572" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E572" s="1">
         <v>0</v>
@@ -12692,10 +12689,10 @@
         <v>515</v>
       </c>
       <c r="C573" s="10" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="D573" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E573" s="1">
         <v>0</v>
@@ -12709,10 +12706,10 @@
         <v>515</v>
       </c>
       <c r="C574" s="10" t="s">
-        <v>682</v>
+        <v>542</v>
       </c>
       <c r="D574" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E574" s="1">
         <v>0</v>
@@ -12726,7 +12723,7 @@
         <v>515</v>
       </c>
       <c r="C575" s="10" t="s">
-        <v>542</v>
+        <v>683</v>
       </c>
       <c r="D575" s="13">
         <v>1</v>
@@ -12743,10 +12740,10 @@
         <v>515</v>
       </c>
       <c r="C576" s="10" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="D576" s="13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E576" s="1">
         <v>0</v>
@@ -12760,10 +12757,10 @@
         <v>515</v>
       </c>
       <c r="C577" s="10" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="D577" s="13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E577" s="1">
         <v>0</v>
@@ -12777,7 +12774,7 @@
         <v>515</v>
       </c>
       <c r="C578" s="10" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="D578" s="13">
         <v>2</v>
@@ -12794,10 +12791,10 @@
         <v>515</v>
       </c>
       <c r="C579" s="10" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="D579" s="13">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E579" s="1">
         <v>0</v>
@@ -12811,7 +12808,7 @@
         <v>515</v>
       </c>
       <c r="C580" s="10" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="D580" s="13">
         <v>4</v>
@@ -12828,10 +12825,10 @@
         <v>515</v>
       </c>
       <c r="C581" s="10" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="D581" s="13">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E581" s="1">
         <v>0</v>
@@ -12845,7 +12842,7 @@
         <v>515</v>
       </c>
       <c r="C582" s="10" t="s">
-        <v>689</v>
+        <v>543</v>
       </c>
       <c r="D582" s="13">
         <v>2</v>
@@ -12862,10 +12859,10 @@
         <v>515</v>
       </c>
       <c r="C583" s="10" t="s">
-        <v>543</v>
+        <v>677</v>
       </c>
       <c r="D583" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E583" s="1">
         <v>0</v>
@@ -12873,13 +12870,13 @@
     </row>
     <row r="584" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A584" s="10" t="s">
-        <v>555</v>
+        <v>611</v>
       </c>
       <c r="B584" s="10" t="s">
         <v>515</v>
       </c>
       <c r="C584" s="10" t="s">
-        <v>677</v>
+        <v>544</v>
       </c>
       <c r="D584" s="13">
         <v>1</v>
@@ -12890,16 +12887,16 @@
     </row>
     <row r="585" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A585" s="10" t="s">
-        <v>611</v>
+        <v>557</v>
       </c>
       <c r="B585" s="10" t="s">
-        <v>515</v>
+        <v>0</v>
       </c>
       <c r="C585" s="10" t="s">
-        <v>544</v>
+        <v>306</v>
       </c>
       <c r="D585" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E585" s="1">
         <v>0</v>
@@ -12907,16 +12904,16 @@
     </row>
     <row r="586" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A586" s="10" t="s">
-        <v>557</v>
+        <v>611</v>
       </c>
       <c r="B586" s="10" t="s">
-        <v>0</v>
+        <v>515</v>
       </c>
       <c r="C586" s="10" t="s">
-        <v>306</v>
+        <v>548</v>
       </c>
       <c r="D586" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E586" s="1">
         <v>0</v>
@@ -12924,16 +12921,16 @@
     </row>
     <row r="587" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A587" s="10" t="s">
-        <v>611</v>
+        <v>633</v>
       </c>
       <c r="B587" s="10" t="s">
-        <v>515</v>
+        <v>39</v>
       </c>
       <c r="C587" s="10" t="s">
-        <v>548</v>
+        <v>398</v>
       </c>
       <c r="D587" s="13">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="E587" s="1">
         <v>0</v>
@@ -12947,10 +12944,10 @@
         <v>39</v>
       </c>
       <c r="C588" s="10" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D588" s="13">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="E588" s="1">
         <v>0</v>
@@ -12958,16 +12955,16 @@
     </row>
     <row r="589" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A589" s="10" t="s">
-        <v>633</v>
+        <v>555</v>
       </c>
       <c r="B589" s="10" t="s">
-        <v>39</v>
+        <v>515</v>
       </c>
       <c r="C589" s="10" t="s">
-        <v>399</v>
+        <v>764</v>
       </c>
       <c r="D589" s="13">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="E589" s="1">
         <v>0</v>
@@ -13001,7 +12998,7 @@
         <v>766</v>
       </c>
       <c r="D591" s="13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E591" s="1">
         <v>0</v>
@@ -13018,7 +13015,7 @@
         <v>767</v>
       </c>
       <c r="D592" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E592" s="1">
         <v>0</v>
@@ -13026,16 +13023,16 @@
     </row>
     <row r="593" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A593" s="10" t="s">
-        <v>555</v>
+        <v>549</v>
       </c>
       <c r="B593" s="10" t="s">
-        <v>515</v>
+        <v>0</v>
       </c>
       <c r="C593" s="10" t="s">
-        <v>768</v>
+        <v>307</v>
       </c>
       <c r="D593" s="13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E593" s="1">
         <v>0</v>
@@ -13043,16 +13040,16 @@
     </row>
     <row r="594" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A594" s="10" t="s">
-        <v>549</v>
+        <v>657</v>
       </c>
       <c r="B594" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C594" s="10" t="s">
-        <v>307</v>
+        <v>779</v>
       </c>
       <c r="D594" s="13">
-        <v>1</v>
+        <v>2000</v>
       </c>
       <c r="E594" s="1">
         <v>0</v>
@@ -13060,7 +13057,7 @@
     </row>
     <row r="595" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A595" s="10" t="s">
-        <v>657</v>
+        <v>652</v>
       </c>
       <c r="B595" s="10" t="s">
         <v>39</v>
@@ -13069,7 +13066,7 @@
         <v>780</v>
       </c>
       <c r="D595" s="13">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="E595" s="1">
         <v>0</v>
@@ -13083,10 +13080,10 @@
         <v>39</v>
       </c>
       <c r="C596" s="10" t="s">
-        <v>781</v>
+        <v>788</v>
       </c>
       <c r="D596" s="13">
-        <v>2500</v>
+        <v>2400</v>
       </c>
       <c r="E596" s="1">
         <v>0</v>
@@ -13094,16 +13091,16 @@
     </row>
     <row r="597" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A597" s="10" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="B597" s="10" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="C597" s="10" t="s">
-        <v>789</v>
+        <v>794</v>
       </c>
       <c r="D597" s="13">
-        <v>2400</v>
+        <v>1</v>
       </c>
       <c r="E597" s="1">
         <v>0</v>
@@ -13120,7 +13117,7 @@
         <v>795</v>
       </c>
       <c r="D598" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E598" s="1">
         <v>0</v>
@@ -13134,10 +13131,10 @@
         <v>9</v>
       </c>
       <c r="C599" s="10" t="s">
-        <v>796</v>
+        <v>423</v>
       </c>
       <c r="D599" s="13">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E599" s="1">
         <v>0</v>
@@ -13151,10 +13148,10 @@
         <v>9</v>
       </c>
       <c r="C600" s="10" t="s">
-        <v>423</v>
+        <v>512</v>
       </c>
       <c r="D600" s="13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E600" s="1">
         <v>0</v>
@@ -13162,16 +13159,16 @@
     </row>
     <row r="601" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A601" s="10" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="B601" s="10" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="C601" s="10" t="s">
-        <v>512</v>
+        <v>781</v>
       </c>
       <c r="D601" s="13">
-        <v>1</v>
+        <v>1850</v>
       </c>
       <c r="E601" s="1">
         <v>0</v>
@@ -13179,16 +13176,16 @@
     </row>
     <row r="602" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A602" s="10" t="s">
-        <v>652</v>
+        <v>657</v>
       </c>
       <c r="B602" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C602" s="10" t="s">
-        <v>782</v>
+        <v>308</v>
       </c>
       <c r="D602" s="13">
-        <v>1850</v>
+        <v>37</v>
       </c>
       <c r="E602" s="1">
         <v>0</v>
@@ -13196,16 +13193,16 @@
     </row>
     <row r="603" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A603" s="10" t="s">
-        <v>657</v>
+        <v>652</v>
       </c>
       <c r="B603" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C603" s="10" t="s">
-        <v>308</v>
+        <v>782</v>
       </c>
       <c r="D603" s="13">
-        <v>37</v>
+        <v>2500</v>
       </c>
       <c r="E603" s="1">
         <v>0</v>
@@ -13219,10 +13216,10 @@
         <v>39</v>
       </c>
       <c r="C604" s="10" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="D604" s="13">
-        <v>2500</v>
+        <v>2400</v>
       </c>
       <c r="E604" s="1">
         <v>0</v>
@@ -13230,16 +13227,16 @@
     </row>
     <row r="605" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A605" s="10" t="s">
-        <v>652</v>
+        <v>657</v>
       </c>
       <c r="B605" s="10" t="s">
         <v>39</v>
       </c>
       <c r="C605" s="10" t="s">
-        <v>790</v>
+        <v>728</v>
       </c>
       <c r="D605" s="13">
-        <v>2400</v>
+        <v>800</v>
       </c>
       <c r="E605" s="1">
         <v>0</v>
@@ -13253,10 +13250,10 @@
         <v>39</v>
       </c>
       <c r="C606" s="10" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="D606" s="13">
-        <v>800</v>
+        <v>1600</v>
       </c>
       <c r="E606" s="1">
         <v>0</v>
@@ -13270,10 +13267,10 @@
         <v>39</v>
       </c>
       <c r="C607" s="10" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="D607" s="13">
-        <v>1600</v>
+        <v>1000</v>
       </c>
       <c r="E607" s="1">
         <v>0</v>
@@ -13287,10 +13284,10 @@
         <v>39</v>
       </c>
       <c r="C608" s="10" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="D608" s="13">
-        <v>1000</v>
+        <v>1600</v>
       </c>
       <c r="E608" s="1">
         <v>0</v>
@@ -13304,10 +13301,10 @@
         <v>39</v>
       </c>
       <c r="C609" s="10" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="D609" s="13">
-        <v>1600</v>
+        <v>800</v>
       </c>
       <c r="E609" s="1">
         <v>0</v>
@@ -13321,10 +13318,10 @@
         <v>39</v>
       </c>
       <c r="C610" s="10" t="s">
-        <v>732</v>
+        <v>783</v>
       </c>
       <c r="D610" s="13">
-        <v>800</v>
+        <v>1250</v>
       </c>
       <c r="E610" s="1">
         <v>0</v>
@@ -13341,7 +13338,7 @@
         <v>784</v>
       </c>
       <c r="D611" s="13">
-        <v>1250</v>
+        <v>1550</v>
       </c>
       <c r="E611" s="1">
         <v>0</v>
@@ -13352,13 +13349,13 @@
         <v>657</v>
       </c>
       <c r="B612" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C612" s="10" t="s">
-        <v>785</v>
+        <v>309</v>
       </c>
       <c r="D612" s="13">
-        <v>1550</v>
+        <v>1070</v>
       </c>
       <c r="E612" s="1">
         <v>0</v>
@@ -13369,13 +13366,13 @@
         <v>657</v>
       </c>
       <c r="B613" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C613" s="10" t="s">
-        <v>309</v>
+        <v>785</v>
       </c>
       <c r="D613" s="13">
-        <v>1070</v>
+        <v>1700</v>
       </c>
       <c r="E613" s="1">
         <v>0</v>
@@ -13392,7 +13389,7 @@
         <v>786</v>
       </c>
       <c r="D614" s="13">
-        <v>1700</v>
+        <v>1000</v>
       </c>
       <c r="E614" s="1">
         <v>0</v>
@@ -13400,16 +13397,16 @@
     </row>
     <row r="615" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A615" s="10" t="s">
-        <v>657</v>
+        <v>565</v>
       </c>
       <c r="B615" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C615" s="10" t="s">
-        <v>787</v>
+        <v>310</v>
       </c>
       <c r="D615" s="13">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="E615" s="1">
         <v>0</v>
@@ -13423,10 +13420,10 @@
         <v>0</v>
       </c>
       <c r="C616" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D616" s="13">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E616" s="1">
         <v>0</v>
@@ -13434,16 +13431,16 @@
     </row>
     <row r="617" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A617" s="10" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B617" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C617" s="10" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D617" s="13">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E617" s="1">
         <v>0</v>
@@ -13457,7 +13454,7 @@
         <v>0</v>
       </c>
       <c r="C618" s="10" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D618" s="13">
         <v>1</v>
@@ -13468,16 +13465,16 @@
     </row>
     <row r="619" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A619" s="10" t="s">
-        <v>566</v>
+        <v>658</v>
       </c>
       <c r="B619" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C619" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D619" s="13">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="E619" s="1">
         <v>0</v>
@@ -13485,16 +13482,16 @@
     </row>
     <row r="620" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A620" s="10" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="B620" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C620" s="10" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D620" s="13">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E620" s="1">
         <v>0</v>
@@ -13508,10 +13505,10 @@
         <v>0</v>
       </c>
       <c r="C621" s="10" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D621" s="13">
-        <v>46</v>
+        <v>121</v>
       </c>
       <c r="E621" s="1">
         <v>0</v>
@@ -13519,16 +13516,16 @@
     </row>
     <row r="622" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A622" s="10" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B622" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C622" s="10" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D622" s="13">
-        <v>121</v>
+        <v>300</v>
       </c>
       <c r="E622" s="1">
         <v>0</v>
@@ -13539,7 +13536,7 @@
         <v>660</v>
       </c>
       <c r="B623" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C623" s="10" t="s">
         <v>317</v>
@@ -13553,13 +13550,13 @@
     </row>
     <row r="624" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A624" s="10" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B624" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C624" s="10" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D624" s="13">
         <v>300</v>
@@ -13570,16 +13567,16 @@
     </row>
     <row r="625" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A625" s="10" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B625" s="10" t="s">
         <v>39</v>
       </c>
       <c r="C625" s="10" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D625" s="13">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="E625" s="1">
         <v>0</v>
@@ -13587,16 +13584,16 @@
     </row>
     <row r="626" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A626" s="10" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="B626" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C626" s="10" t="s">
-        <v>319</v>
+        <v>447</v>
       </c>
       <c r="D626" s="13">
-        <v>310</v>
+        <v>43</v>
       </c>
       <c r="E626" s="1">
         <v>0</v>
@@ -13604,16 +13601,16 @@
     </row>
     <row r="627" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A627" s="10" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B627" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C627" s="10" t="s">
-        <v>447</v>
+        <v>320</v>
       </c>
       <c r="D627" s="13">
-        <v>43</v>
+        <v>250</v>
       </c>
       <c r="E627" s="1">
         <v>0</v>
@@ -13624,13 +13621,13 @@
         <v>661</v>
       </c>
       <c r="B628" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C628" s="10" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D628" s="13">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="E628" s="1">
         <v>0</v>
@@ -13641,13 +13638,13 @@
         <v>661</v>
       </c>
       <c r="B629" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C629" s="10" t="s">
         <v>321</v>
       </c>
       <c r="D629" s="13">
-        <v>300</v>
+        <v>280</v>
       </c>
       <c r="E629" s="1">
         <v>0</v>
@@ -13658,13 +13655,13 @@
         <v>661</v>
       </c>
       <c r="B630" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C630" s="10" t="s">
-        <v>321</v>
+        <v>393</v>
       </c>
       <c r="D630" s="13">
-        <v>280</v>
+        <v>42</v>
       </c>
       <c r="E630" s="1">
         <v>0</v>
@@ -13678,10 +13675,10 @@
         <v>39</v>
       </c>
       <c r="C631" s="10" t="s">
-        <v>393</v>
+        <v>322</v>
       </c>
       <c r="D631" s="13">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="E631" s="1">
         <v>0</v>
@@ -13689,16 +13686,16 @@
     </row>
     <row r="632" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A632" s="10" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="B632" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C632" s="10" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D632" s="13">
-        <v>24</v>
+        <v>250</v>
       </c>
       <c r="E632" s="1">
         <v>0</v>
@@ -13706,16 +13703,16 @@
     </row>
     <row r="633" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A633" s="10" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B633" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C633" s="10" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D633" s="13">
-        <v>250</v>
+        <v>1250</v>
       </c>
       <c r="E633" s="1">
         <v>0</v>
@@ -13723,16 +13720,16 @@
     </row>
     <row r="634" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A634" s="10" t="s">
-        <v>664</v>
+        <v>719</v>
       </c>
       <c r="B634" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C634" s="10" t="s">
-        <v>324</v>
+        <v>720</v>
       </c>
       <c r="D634" s="13">
-        <v>1250</v>
+        <v>100</v>
       </c>
       <c r="E634" s="1">
         <v>0</v>
@@ -13740,16 +13737,16 @@
     </row>
     <row r="635" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A635" s="10" t="s">
-        <v>719</v>
+        <v>664</v>
       </c>
       <c r="B635" s="10" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C635" s="10" t="s">
-        <v>720</v>
+        <v>325</v>
       </c>
       <c r="D635" s="13">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="E635" s="1">
         <v>0</v>
@@ -13757,16 +13754,16 @@
     </row>
     <row r="636" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A636" s="10" t="s">
-        <v>664</v>
+        <v>719</v>
       </c>
       <c r="B636" s="10" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C636" s="10" t="s">
-        <v>325</v>
+        <v>721</v>
       </c>
       <c r="D636" s="13">
-        <v>160</v>
+        <v>35</v>
       </c>
       <c r="E636" s="1">
         <v>0</v>
@@ -13774,16 +13771,16 @@
     </row>
     <row r="637" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A637" s="10" t="s">
-        <v>719</v>
+        <v>664</v>
       </c>
       <c r="B637" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C637" s="10" t="s">
-        <v>721</v>
+        <v>326</v>
       </c>
       <c r="D637" s="13">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="E637" s="1">
         <v>0</v>
@@ -13808,16 +13805,16 @@
     </row>
     <row r="639" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A639" s="1" t="s">
-        <v>664</v>
+        <v>719</v>
       </c>
       <c r="B639" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C639" s="1" t="s">
-        <v>326</v>
+        <v>722</v>
       </c>
       <c r="D639" s="14">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="E639" s="1">
         <v>0</v>
@@ -13825,16 +13822,16 @@
     </row>
     <row r="640" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A640" s="1" t="s">
-        <v>719</v>
+        <v>664</v>
       </c>
       <c r="B640" s="1" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C640" s="1" t="s">
-        <v>722</v>
+        <v>391</v>
       </c>
       <c r="D640" s="14">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="E640" s="1">
         <v>0</v>
@@ -13848,10 +13845,10 @@
         <v>39</v>
       </c>
       <c r="C641" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D641" s="14">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="E641" s="1">
         <v>0</v>
@@ -13865,10 +13862,10 @@
         <v>39</v>
       </c>
       <c r="C642" s="1" t="s">
-        <v>392</v>
+        <v>327</v>
       </c>
       <c r="D642" s="14">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="E642" s="1">
         <v>0</v>
@@ -13876,16 +13873,16 @@
     </row>
     <row r="643" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A643" s="1" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B643" s="1" t="s">
-        <v>39</v>
+        <v>405</v>
       </c>
       <c r="C643" s="1" t="s">
-        <v>327</v>
+        <v>416</v>
       </c>
       <c r="D643" s="14">
-        <v>72</v>
+        <v>2</v>
       </c>
       <c r="E643" s="1">
         <v>0</v>
@@ -13896,13 +13893,13 @@
         <v>665</v>
       </c>
       <c r="B644" s="1" t="s">
-        <v>405</v>
+        <v>0</v>
       </c>
       <c r="C644" s="1" t="s">
-        <v>416</v>
+        <v>328</v>
       </c>
       <c r="D644" s="14">
-        <v>2</v>
+        <v>1300</v>
       </c>
       <c r="E644" s="1">
         <v>0</v>
@@ -13916,10 +13913,10 @@
         <v>0</v>
       </c>
       <c r="C645" s="1" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D645" s="14">
-        <v>1300</v>
+        <v>29</v>
       </c>
       <c r="E645" s="1">
         <v>0</v>
@@ -13933,10 +13930,10 @@
         <v>0</v>
       </c>
       <c r="C646" s="1" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D646" s="14">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="E646" s="1">
         <v>0</v>
@@ -13944,16 +13941,16 @@
     </row>
     <row r="647" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A647" s="1" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B647" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C647" s="1" t="s">
-        <v>330</v>
+        <v>464</v>
       </c>
       <c r="D647" s="14">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E647" s="1">
         <v>0</v>
@@ -13967,10 +13964,10 @@
         <v>0</v>
       </c>
       <c r="C648" s="1" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D648" s="14">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E648" s="1">
         <v>0</v>
@@ -13984,10 +13981,10 @@
         <v>0</v>
       </c>
       <c r="C649" s="1" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D649" s="14">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E649" s="1">
         <v>0</v>
@@ -13995,16 +13992,16 @@
     </row>
     <row r="650" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A650" s="1" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B650" s="1" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C650" s="1" t="s">
-        <v>466</v>
+        <v>331</v>
       </c>
       <c r="D650" s="14">
-        <v>4</v>
+        <v>72</v>
       </c>
       <c r="E650" s="1">
         <v>0</v>
@@ -14018,10 +14015,10 @@
         <v>9</v>
       </c>
       <c r="C651" s="1" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D651" s="14">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="E651" s="1">
         <v>0</v>
@@ -14035,10 +14032,10 @@
         <v>9</v>
       </c>
       <c r="C652" s="1" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D652" s="14">
-        <v>78</v>
+        <v>8</v>
       </c>
       <c r="E652" s="1">
         <v>0</v>
@@ -14052,10 +14049,10 @@
         <v>9</v>
       </c>
       <c r="C653" s="1" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D653" s="14">
-        <v>8</v>
+        <v>200</v>
       </c>
       <c r="E653" s="1">
         <v>0</v>
@@ -14063,16 +14060,16 @@
     </row>
     <row r="654" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A654" s="1" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B654" s="1" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="C654" s="1" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D654" s="14">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="E654" s="1">
         <v>0</v>
@@ -14086,10 +14083,10 @@
         <v>39</v>
       </c>
       <c r="C655" s="1" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D655" s="14">
-        <v>600</v>
+        <v>825</v>
       </c>
       <c r="E655" s="1">
         <v>0</v>
@@ -14097,16 +14094,16 @@
     </row>
     <row r="656" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A656" s="1" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="B656" s="1" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C656" s="1" t="s">
-        <v>336</v>
+        <v>723</v>
       </c>
       <c r="D656" s="14">
-        <v>825</v>
+        <v>465</v>
       </c>
       <c r="E656" s="1">
         <v>0</v>
@@ -14114,16 +14111,16 @@
     </row>
     <row r="657" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A657" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B657" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C657" s="1" t="s">
-        <v>723</v>
+        <v>337</v>
       </c>
       <c r="D657" s="14">
-        <v>465</v>
+        <v>400</v>
       </c>
       <c r="E657" s="1">
         <v>0</v>
@@ -14148,16 +14145,16 @@
     </row>
     <row r="659" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A659" s="1" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B659" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C659" s="1" t="s">
-        <v>337</v>
+        <v>448</v>
       </c>
       <c r="D659" s="14">
-        <v>400</v>
+        <v>65</v>
       </c>
       <c r="E659" s="1">
         <v>0</v>
@@ -14165,16 +14162,16 @@
     </row>
     <row r="660" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A660" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B660" s="1" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C660" s="1" t="s">
-        <v>448</v>
+        <v>377</v>
       </c>
       <c r="D660" s="14">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="E660" s="1">
         <v>0</v>
@@ -14188,10 +14185,10 @@
         <v>39</v>
       </c>
       <c r="C661" s="1" t="s">
-        <v>377</v>
+        <v>338</v>
       </c>
       <c r="D661" s="14">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="E661" s="1">
         <v>0</v>
@@ -14199,16 +14196,16 @@
     </row>
     <row r="662" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A662" s="1" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="B662" s="1" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C662" s="1" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D662" s="14">
-        <v>72</v>
+        <v>1001</v>
       </c>
       <c r="E662" s="1">
         <v>0</v>
@@ -14222,10 +14219,10 @@
         <v>0</v>
       </c>
       <c r="C663" s="1" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D663" s="14">
-        <v>1001</v>
+        <v>1508</v>
       </c>
       <c r="E663" s="1">
         <v>0</v>
@@ -14233,16 +14230,16 @@
     </row>
     <row r="664" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A664" s="1" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B664" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C664" s="1" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D664" s="14">
-        <v>1508</v>
+        <v>600</v>
       </c>
       <c r="E664" s="1">
         <v>0</v>
@@ -14256,10 +14253,10 @@
         <v>0</v>
       </c>
       <c r="C665" s="1" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D665" s="14">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="E665" s="1">
         <v>0</v>
@@ -14273,10 +14270,10 @@
         <v>0</v>
       </c>
       <c r="C666" s="1" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D666" s="14">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E666" s="1">
         <v>0</v>
@@ -14290,10 +14287,10 @@
         <v>0</v>
       </c>
       <c r="C667" s="1" t="s">
-        <v>343</v>
+        <v>500</v>
       </c>
       <c r="D667" s="14">
-        <v>300</v>
+        <v>1000</v>
       </c>
       <c r="E667" s="1">
         <v>0</v>
@@ -14307,10 +14304,10 @@
         <v>0</v>
       </c>
       <c r="C668" s="1" t="s">
-        <v>500</v>
+        <v>344</v>
       </c>
       <c r="D668" s="14">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="E668" s="1">
         <v>0</v>
@@ -14324,7 +14321,7 @@
         <v>0</v>
       </c>
       <c r="C669" s="1" t="s">
-        <v>344</v>
+        <v>404</v>
       </c>
       <c r="D669" s="14">
         <v>100</v>
@@ -14341,10 +14338,10 @@
         <v>0</v>
       </c>
       <c r="C670" s="1" t="s">
-        <v>404</v>
+        <v>345</v>
       </c>
       <c r="D670" s="14">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="E670" s="1">
         <v>0</v>
@@ -14352,16 +14349,16 @@
     </row>
     <row r="671" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A671" s="1" t="s">
-        <v>672</v>
+        <v>658</v>
       </c>
       <c r="B671" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C671" s="1" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D671" s="14">
-        <v>500</v>
+        <v>170</v>
       </c>
       <c r="E671" s="1">
         <v>0</v>
@@ -14375,10 +14372,10 @@
         <v>0</v>
       </c>
       <c r="C672" s="1" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D672" s="14">
-        <v>170</v>
+        <v>90</v>
       </c>
       <c r="E672" s="1">
         <v>0</v>
@@ -14386,16 +14383,16 @@
     </row>
     <row r="673" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A673" s="1" t="s">
-        <v>658</v>
+        <v>673</v>
       </c>
       <c r="B673" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C673" s="1" t="s">
-        <v>347</v>
+        <v>467</v>
       </c>
       <c r="D673" s="14">
-        <v>90</v>
+        <v>13</v>
       </c>
       <c r="E673" s="1">
         <v>0</v>
@@ -14409,10 +14406,10 @@
         <v>0</v>
       </c>
       <c r="C674" s="1" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D674" s="14">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E674" s="1">
         <v>0</v>
@@ -14426,10 +14423,10 @@
         <v>0</v>
       </c>
       <c r="C675" s="1" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D675" s="14">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E675" s="1">
         <v>0</v>
@@ -14437,16 +14434,16 @@
     </row>
     <row r="676" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A676" s="1" t="s">
-        <v>673</v>
+        <v>659</v>
       </c>
       <c r="B676" s="1" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C676" s="1" t="s">
-        <v>469</v>
+        <v>348</v>
       </c>
       <c r="D676" s="14">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E676" s="1">
         <v>0</v>
@@ -14460,10 +14457,10 @@
         <v>9</v>
       </c>
       <c r="C677" s="1" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D677" s="14">
-        <v>15</v>
+        <v>225</v>
       </c>
       <c r="E677" s="1">
         <v>0</v>
@@ -14477,10 +14474,10 @@
         <v>9</v>
       </c>
       <c r="C678" s="1" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D678" s="14">
-        <v>225</v>
+        <v>150</v>
       </c>
       <c r="E678" s="1">
         <v>0</v>
@@ -14488,16 +14485,16 @@
     </row>
     <row r="679" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A679" s="1" t="s">
-        <v>659</v>
+        <v>674</v>
       </c>
       <c r="B679" s="1" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C679" s="1" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D679" s="14">
-        <v>150</v>
+        <v>1200</v>
       </c>
       <c r="E679" s="1">
         <v>0</v>
@@ -14508,10 +14505,10 @@
         <v>674</v>
       </c>
       <c r="B680" s="1" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C680" s="1" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D680" s="14">
         <v>1200</v>
@@ -14528,10 +14525,10 @@
         <v>39</v>
       </c>
       <c r="C681" s="1" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D681" s="14">
-        <v>1200</v>
+        <v>300</v>
       </c>
       <c r="E681" s="1">
         <v>0</v>
@@ -14562,10 +14559,10 @@
         <v>39</v>
       </c>
       <c r="C683" s="1" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D683" s="14">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="E683" s="1">
         <v>0</v>
@@ -14573,16 +14570,16 @@
     </row>
     <row r="684" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A684" s="1" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B684" s="1" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C684" s="1" t="s">
-        <v>354</v>
+        <v>748</v>
       </c>
       <c r="D684" s="14">
-        <v>500</v>
+        <v>235</v>
       </c>
       <c r="E684" s="1">
         <v>0</v>
@@ -14596,10 +14593,10 @@
         <v>0</v>
       </c>
       <c r="C685" s="1" t="s">
-        <v>748</v>
+        <v>724</v>
       </c>
       <c r="D685" s="14">
-        <v>235</v>
+        <v>150</v>
       </c>
       <c r="E685" s="1">
         <v>0</v>
@@ -14607,16 +14604,16 @@
     </row>
     <row r="686" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A686" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B686" s="1" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C686" s="1" t="s">
-        <v>724</v>
+        <v>355</v>
       </c>
       <c r="D686" s="14">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="E686" s="1">
         <v>0</v>
@@ -14644,13 +14641,13 @@
         <v>674</v>
       </c>
       <c r="B688" s="1" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C688" s="1" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D688" s="14">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="E688" s="1">
         <v>0</v>
@@ -14664,10 +14661,10 @@
         <v>0</v>
       </c>
       <c r="C689" s="1" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D689" s="14">
-        <v>175</v>
+        <v>225</v>
       </c>
       <c r="E689" s="1">
         <v>0</v>
@@ -14675,16 +14672,16 @@
     </row>
     <row r="690" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A690" s="1" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B690" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C690" s="1" t="s">
-        <v>357</v>
+        <v>449</v>
       </c>
       <c r="D690" s="14">
-        <v>225</v>
+        <v>10</v>
       </c>
       <c r="E690" s="1">
         <v>0</v>
@@ -14692,16 +14689,16 @@
     </row>
     <row r="691" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A691" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B691" s="1" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C691" s="1" t="s">
-        <v>449</v>
+        <v>358</v>
       </c>
       <c r="D691" s="14">
-        <v>10</v>
+        <v>125</v>
       </c>
       <c r="E691" s="1">
         <v>0</v>
@@ -14729,13 +14726,13 @@
         <v>674</v>
       </c>
       <c r="B693" s="1" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C693" s="1" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D693" s="14">
-        <v>125</v>
+        <v>94</v>
       </c>
       <c r="E693" s="1">
         <v>0</v>
@@ -14746,13 +14743,13 @@
         <v>674</v>
       </c>
       <c r="B694" s="1" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C694" s="1" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D694" s="14">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="E694" s="1">
         <v>0</v>
@@ -14763,13 +14760,13 @@
         <v>674</v>
       </c>
       <c r="B695" s="1" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C695" s="1" t="s">
         <v>360</v>
       </c>
       <c r="D695" s="14">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="E695" s="1">
         <v>0</v>
@@ -14780,13 +14777,13 @@
         <v>674</v>
       </c>
       <c r="B696" s="1" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C696" s="1" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D696" s="14">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E696" s="1">
         <v>0</v>
@@ -14806,23 +14803,6 @@
         <v>30</v>
       </c>
       <c r="E697" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="698" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A698" s="1" t="s">
-        <v>674</v>
-      </c>
-      <c r="B698" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C698" s="1" t="s">
-        <v>361</v>
-      </c>
-      <c r="D698" s="14">
-        <v>64</v>
-      </c>
-      <c r="E698" s="1">
         <v>0</v>
       </c>
     </row>
@@ -14889,11 +14869,11 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="str" cm="1">
-        <f t="array" ref="A6:C9">_xlfn._xlws.SORT(_xlfn._xlws.FILTER('جرد المواد'!B5:D9560,
-ISNUMBER(SEARCH(IF(B1="","*",B1),'جرد المواد'!C5:C9560))*
-ISNUMBER(SEARCH(IF(B2="","*",B2),'جرد المواد'!C5:C9560))*
-ISNUMBER(SEARCH(IF(B3="","*",B3),'جرد المواد'!C5:C9560))*
-ISNUMBER(SEARCH(IF(B4="","*",B4),'جرد المواد'!B5:B9560)),
+        <f t="array" ref="A6:C9">_xlfn._xlws.SORT(_xlfn._xlws.FILTER('جرد المواد'!B5:D9559,
+ISNUMBER(SEARCH(IF(B1="","*",B1),'جرد المواد'!C5:C9559))*
+ISNUMBER(SEARCH(IF(B2="","*",B2),'جرد المواد'!C5:C9559))*
+ISNUMBER(SEARCH(IF(B3="","*",B3),'جرد المواد'!C5:C9559))*
+ISNUMBER(SEARCH(IF(B4="","*",B4),'جرد المواد'!B5:B9559)),
 "لا توجد نتائج"),
 2,1)</f>
         <v>3-ديوان</v>

</xml_diff>